<commit_message>
Export fixes: Avg General column + Read me variant count
- Company averages sheet: add Avg General (0-100) between Avg G and
  Avg Composite; extend color-scale range to cover all five score cols
- Read me sheet: correct 'four variants' to 'seven variants' (the
  Robustness sheet has 3-pillar, no-new-3, w=1.0, w=1.25, w=2.0,
  sector-adjusted, without-5)
- Regenerated xlsx and csv (390 rows, 65 companies, pipeline 0.6.0)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/verity_esg_scores.xlsx
+++ b/docs/exports/verity_esg_scores.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scores by year'!$A$1:$Y$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Company averages'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Company averages'!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -516,98 +516,105 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Terms material to a company's SASB industry are weighted 1.5; others 1.0.</t>
+          <t>Term concepts: E=24, S=22 (27 phrases), G=34 (36 phrases), General=8, Banking add-on=9.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Scores are rank-normalised 0–100 across all 390 reports; 100 = most disclosure.</t>
+          <t>Terms material to a company's SASB industry are weighted 1.5; others 1.0.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Scores are rank-normalised 0-100 across all 390 reports; 100 = most disclosure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Composite = average of Environmental, Social, Governance, and General scores.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>How to read a 0–100 score</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>100 = the report with the most disclosure in this sample for that pillar.</t>
+          <t>How to read a 0–100 score</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0   = the report with the least.</t>
+          <t>100 = the report with the most disclosure in this sample for that pillar.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>0   = the report with the least.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Scores show relative position within this sample, not absolute quality.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Methodology page: see the Verity web dashboard → Methodology.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Sheets</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Scores by year   — one row per company-year</t>
+          <t>Sheets</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Company averages — six-year averages, ranked 1–65</t>
+          <t>Scores by year   — one row per company-year</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Robustness       — main composite vs four variants + correlations</t>
+          <t>Company averages — six-year averages, ranked 1–65</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
+        <is>
+          <t>Robustness       — main composite vs seven variants + correlations</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Column guide     — definition and unit of every column</t>
         </is>
@@ -34211,7 +34218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -34224,8 +34231,9 @@
     <col width="27" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -34281,10 +34289,15 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
+          <t>Avg General (0-100)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
           <t>Avg Composite (0-100)</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Years scored</t>
         </is>
@@ -34334,9 +34347,12 @@
         <v>55.38</v>
       </c>
       <c r="K2" t="n">
+        <v>90.15000000000001</v>
+      </c>
+      <c r="L2" t="n">
         <v>74.92</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34384,9 +34400,12 @@
         <v>68.77</v>
       </c>
       <c r="K3" s="4" t="n">
+        <v>81.72</v>
+      </c>
+      <c r="L3" s="4" t="n">
         <v>72.08</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34434,9 +34453,12 @@
         <v>75.65000000000001</v>
       </c>
       <c r="K4" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="L4" t="n">
         <v>69.15000000000001</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34484,9 +34506,12 @@
         <v>76.37</v>
       </c>
       <c r="K5" s="4" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>68.45</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34534,9 +34559,12 @@
         <v>20.18</v>
       </c>
       <c r="K6" t="n">
+        <v>81.72</v>
+      </c>
+      <c r="L6" t="n">
         <v>68.45</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34584,9 +34612,12 @@
         <v>60.47</v>
       </c>
       <c r="K7" s="4" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34634,9 +34665,12 @@
         <v>56.28</v>
       </c>
       <c r="K8" t="n">
+        <v>67.78</v>
+      </c>
+      <c r="L8" t="n">
         <v>64.81999999999999</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34684,9 +34718,12 @@
         <v>87.34999999999999</v>
       </c>
       <c r="K9" s="4" t="n">
+        <v>72.92</v>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>64.06999999999999</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34734,9 +34771,12 @@
         <v>62.08</v>
       </c>
       <c r="K10" t="n">
+        <v>81.38</v>
+      </c>
+      <c r="L10" t="n">
         <v>63.85</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34784,9 +34824,12 @@
         <v>23.97</v>
       </c>
       <c r="K11" s="4" t="n">
+        <v>70.62</v>
+      </c>
+      <c r="L11" s="4" t="n">
         <v>63.42</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34834,9 +34877,12 @@
         <v>16.03</v>
       </c>
       <c r="K12" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="L12" t="n">
         <v>61.22</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34884,9 +34930,12 @@
         <v>22.4</v>
       </c>
       <c r="K13" s="4" t="n">
+        <v>68.33</v>
+      </c>
+      <c r="L13" s="4" t="n">
         <v>60.85</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34934,9 +34983,12 @@
         <v>94.53</v>
       </c>
       <c r="K14" t="n">
+        <v>8.07</v>
+      </c>
+      <c r="L14" t="n">
         <v>60.3</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>6</v>
       </c>
     </row>
@@ -34984,9 +35036,12 @@
         <v>78.37</v>
       </c>
       <c r="K15" s="4" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="L15" s="4" t="n">
         <v>60.15</v>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="M15" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35034,9 +35089,12 @@
         <v>33.08</v>
       </c>
       <c r="K16" t="n">
+        <v>67.92</v>
+      </c>
+      <c r="L16" t="n">
         <v>60.13</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35084,9 +35142,12 @@
         <v>33.17</v>
       </c>
       <c r="K17" s="4" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="L17" s="4" t="n">
         <v>59.07</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="M17" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35134,9 +35195,12 @@
         <v>49.65</v>
       </c>
       <c r="K18" t="n">
+        <v>67.33</v>
+      </c>
+      <c r="L18" t="n">
         <v>58.73</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35184,9 +35248,12 @@
         <v>90.81999999999999</v>
       </c>
       <c r="K19" s="4" t="n">
+        <v>24.03</v>
+      </c>
+      <c r="L19" s="4" t="n">
         <v>58.72</v>
       </c>
-      <c r="L19" s="4" t="n">
+      <c r="M19" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35234,9 +35301,12 @@
         <v>86.09999999999999</v>
       </c>
       <c r="K20" t="n">
+        <v>41.13</v>
+      </c>
+      <c r="L20" t="n">
         <v>58.58</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35284,9 +35354,12 @@
         <v>44.48</v>
       </c>
       <c r="K21" s="4" t="n">
+        <v>52.58</v>
+      </c>
+      <c r="L21" s="4" t="n">
         <v>58.12</v>
       </c>
-      <c r="L21" s="4" t="n">
+      <c r="M21" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35334,9 +35407,12 @@
         <v>75.02</v>
       </c>
       <c r="K22" t="n">
+        <v>40.88</v>
+      </c>
+      <c r="L22" t="n">
         <v>57.85</v>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35384,9 +35460,12 @@
         <v>45.3</v>
       </c>
       <c r="K23" s="4" t="n">
+        <v>64.98</v>
+      </c>
+      <c r="L23" s="4" t="n">
         <v>57.83</v>
       </c>
-      <c r="L23" s="4" t="n">
+      <c r="M23" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35434,9 +35513,12 @@
         <v>40.02</v>
       </c>
       <c r="K24" t="n">
+        <v>58.02</v>
+      </c>
+      <c r="L24" t="n">
         <v>57.78</v>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35484,9 +35566,12 @@
         <v>29.42</v>
       </c>
       <c r="K25" s="4" t="n">
+        <v>68.15000000000001</v>
+      </c>
+      <c r="L25" s="4" t="n">
         <v>57.1</v>
       </c>
-      <c r="L25" s="4" t="n">
+      <c r="M25" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35534,9 +35619,12 @@
         <v>60.47</v>
       </c>
       <c r="K26" t="n">
+        <v>52.35</v>
+      </c>
+      <c r="L26" t="n">
         <v>56.4</v>
       </c>
-      <c r="L26" t="n">
+      <c r="M26" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35584,9 +35672,12 @@
         <v>50.8</v>
       </c>
       <c r="K27" s="4" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="L27" s="4" t="n">
         <v>55.82</v>
       </c>
-      <c r="L27" s="4" t="n">
+      <c r="M27" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35634,9 +35725,12 @@
         <v>19.38</v>
       </c>
       <c r="K28" t="n">
+        <v>78.15000000000001</v>
+      </c>
+      <c r="L28" t="n">
         <v>55.32</v>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35684,9 +35778,12 @@
         <v>40.25</v>
       </c>
       <c r="K29" s="4" t="n">
+        <v>77.05</v>
+      </c>
+      <c r="L29" s="4" t="n">
         <v>55.2</v>
       </c>
-      <c r="L29" s="4" t="n">
+      <c r="M29" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35734,9 +35831,12 @@
         <v>53.87</v>
       </c>
       <c r="K30" t="n">
+        <v>68.52</v>
+      </c>
+      <c r="L30" t="n">
         <v>55.17</v>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35784,9 +35884,12 @@
         <v>69.18000000000001</v>
       </c>
       <c r="K31" s="4" t="n">
+        <v>58.78</v>
+      </c>
+      <c r="L31" s="4" t="n">
         <v>54.93</v>
       </c>
-      <c r="L31" s="4" t="n">
+      <c r="M31" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35834,9 +35937,12 @@
         <v>80.65000000000001</v>
       </c>
       <c r="K32" t="n">
+        <v>21.53</v>
+      </c>
+      <c r="L32" t="n">
         <v>54.73</v>
       </c>
-      <c r="L32" t="n">
+      <c r="M32" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35884,9 +35990,12 @@
         <v>22.75</v>
       </c>
       <c r="K33" s="4" t="n">
+        <v>72.63</v>
+      </c>
+      <c r="L33" s="4" t="n">
         <v>53.38</v>
       </c>
-      <c r="L33" s="4" t="n">
+      <c r="M33" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35934,9 +36043,12 @@
         <v>53.37</v>
       </c>
       <c r="K34" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="L34" t="n">
         <v>52.33</v>
       </c>
-      <c r="L34" t="n">
+      <c r="M34" t="n">
         <v>6</v>
       </c>
     </row>
@@ -35984,9 +36096,12 @@
         <v>53.05</v>
       </c>
       <c r="K35" s="4" t="n">
+        <v>58.97</v>
+      </c>
+      <c r="L35" s="4" t="n">
         <v>51.9</v>
       </c>
-      <c r="L35" s="4" t="n">
+      <c r="M35" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36034,9 +36149,12 @@
         <v>73.81999999999999</v>
       </c>
       <c r="K36" t="n">
+        <v>34.15</v>
+      </c>
+      <c r="L36" t="n">
         <v>50.98</v>
       </c>
-      <c r="L36" t="n">
+      <c r="M36" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36084,9 +36202,12 @@
         <v>10.72</v>
       </c>
       <c r="K37" s="4" t="n">
+        <v>44.37</v>
+      </c>
+      <c r="L37" s="4" t="n">
         <v>50.52</v>
       </c>
-      <c r="L37" s="4" t="n">
+      <c r="M37" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36134,9 +36255,12 @@
         <v>59.72</v>
       </c>
       <c r="K38" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="L38" t="n">
         <v>50.33</v>
       </c>
-      <c r="L38" t="n">
+      <c r="M38" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36184,9 +36308,12 @@
         <v>32.15</v>
       </c>
       <c r="K39" s="4" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="L39" s="4" t="n">
         <v>48.95</v>
       </c>
-      <c r="L39" s="4" t="n">
+      <c r="M39" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36234,9 +36361,12 @@
         <v>41.03</v>
       </c>
       <c r="K40" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="L40" t="n">
         <v>48.57</v>
       </c>
-      <c r="L40" t="n">
+      <c r="M40" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36284,9 +36414,12 @@
         <v>13.07</v>
       </c>
       <c r="K41" s="4" t="n">
+        <v>70.53</v>
+      </c>
+      <c r="L41" s="4" t="n">
         <v>47.72</v>
       </c>
-      <c r="L41" s="4" t="n">
+      <c r="M41" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36334,9 +36467,12 @@
         <v>24.85</v>
       </c>
       <c r="K42" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="L42" t="n">
         <v>47.67</v>
       </c>
-      <c r="L42" t="n">
+      <c r="M42" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36384,9 +36520,12 @@
         <v>73.25</v>
       </c>
       <c r="K43" s="4" t="n">
+        <v>31.65</v>
+      </c>
+      <c r="L43" s="4" t="n">
         <v>47.57</v>
       </c>
-      <c r="L43" s="4" t="n">
+      <c r="M43" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36434,9 +36573,12 @@
         <v>70.48</v>
       </c>
       <c r="K44" t="n">
+        <v>36.63</v>
+      </c>
+      <c r="L44" t="n">
         <v>47.53</v>
       </c>
-      <c r="L44" t="n">
+      <c r="M44" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36484,9 +36626,12 @@
         <v>78.18000000000001</v>
       </c>
       <c r="K45" s="4" t="n">
+        <v>39.92</v>
+      </c>
+      <c r="L45" s="4" t="n">
         <v>45.72</v>
       </c>
-      <c r="L45" s="4" t="n">
+      <c r="M45" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36534,9 +36679,12 @@
         <v>37.82</v>
       </c>
       <c r="K46" t="n">
+        <v>65.33</v>
+      </c>
+      <c r="L46" t="n">
         <v>45.4</v>
       </c>
-      <c r="L46" t="n">
+      <c r="M46" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36584,9 +36732,12 @@
         <v>58.97</v>
       </c>
       <c r="K47" s="4" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="L47" s="4" t="n">
         <v>44.17</v>
       </c>
-      <c r="L47" s="4" t="n">
+      <c r="M47" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36634,9 +36785,12 @@
         <v>28.72</v>
       </c>
       <c r="K48" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="L48" t="n">
         <v>42.85</v>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36684,9 +36838,12 @@
         <v>26.23</v>
       </c>
       <c r="K49" s="4" t="n">
+        <v>56.25</v>
+      </c>
+      <c r="L49" s="4" t="n">
         <v>41.45</v>
       </c>
-      <c r="L49" s="4" t="n">
+      <c r="M49" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36734,9 +36891,12 @@
         <v>29.95</v>
       </c>
       <c r="K50" t="n">
+        <v>62.08</v>
+      </c>
+      <c r="L50" t="n">
         <v>41.37</v>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36784,9 +36944,12 @@
         <v>75.77</v>
       </c>
       <c r="K51" s="4" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="L51" s="4" t="n">
         <v>41.25</v>
       </c>
-      <c r="L51" s="4" t="n">
+      <c r="M51" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36834,9 +36997,12 @@
         <v>54.23</v>
       </c>
       <c r="K52" t="n">
+        <v>34.63</v>
+      </c>
+      <c r="L52" t="n">
         <v>39.92</v>
       </c>
-      <c r="L52" t="n">
+      <c r="M52" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36884,9 +37050,12 @@
         <v>95.77</v>
       </c>
       <c r="K53" s="4" t="n">
+        <v>18.53</v>
+      </c>
+      <c r="L53" s="4" t="n">
         <v>39.82</v>
       </c>
-      <c r="L53" s="4" t="n">
+      <c r="M53" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36934,9 +37103,12 @@
         <v>59.42</v>
       </c>
       <c r="K54" t="n">
+        <v>69.28</v>
+      </c>
+      <c r="L54" t="n">
         <v>38.27</v>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>6</v>
       </c>
     </row>
@@ -36984,9 +37156,12 @@
         <v>31.15</v>
       </c>
       <c r="K55" s="4" t="n">
+        <v>20.23</v>
+      </c>
+      <c r="L55" s="4" t="n">
         <v>35.82</v>
       </c>
-      <c r="L55" s="4" t="n">
+      <c r="M55" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37034,9 +37209,12 @@
         <v>23.82</v>
       </c>
       <c r="K56" t="n">
+        <v>32.53</v>
+      </c>
+      <c r="L56" t="n">
         <v>35.08</v>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37084,9 +37262,12 @@
         <v>48.75</v>
       </c>
       <c r="K57" s="4" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="L57" s="4" t="n">
         <v>34.02</v>
       </c>
-      <c r="L57" s="4" t="n">
+      <c r="M57" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37134,9 +37315,12 @@
         <v>23.87</v>
       </c>
       <c r="K58" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="L58" t="n">
         <v>32.17</v>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37184,9 +37368,12 @@
         <v>99.34999999999999</v>
       </c>
       <c r="K59" s="4" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="L59" s="4" t="n">
         <v>31.67</v>
       </c>
-      <c r="L59" s="4" t="n">
+      <c r="M59" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37234,9 +37421,12 @@
         <v>14.25</v>
       </c>
       <c r="K60" t="n">
+        <v>30.27</v>
+      </c>
+      <c r="L60" t="n">
         <v>29.92</v>
       </c>
-      <c r="L60" t="n">
+      <c r="M60" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37284,9 +37474,12 @@
         <v>26.63</v>
       </c>
       <c r="K61" s="4" t="n">
+        <v>33.02</v>
+      </c>
+      <c r="L61" s="4" t="n">
         <v>29.78</v>
       </c>
-      <c r="L61" s="4" t="n">
+      <c r="M61" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37334,9 +37527,12 @@
         <v>37.18</v>
       </c>
       <c r="K62" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="L62" t="n">
         <v>27.4</v>
       </c>
-      <c r="L62" t="n">
+      <c r="M62" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37384,9 +37580,12 @@
         <v>52.78</v>
       </c>
       <c r="K63" s="4" t="n">
+        <v>20.15</v>
+      </c>
+      <c r="L63" s="4" t="n">
         <v>27.25</v>
       </c>
-      <c r="L63" s="4" t="n">
+      <c r="M63" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37434,9 +37633,12 @@
         <v>78.78</v>
       </c>
       <c r="K64" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="L64" t="n">
         <v>26.6</v>
       </c>
-      <c r="L64" t="n">
+      <c r="M64" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37484,9 +37686,12 @@
         <v>13.03</v>
       </c>
       <c r="K65" s="4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="L65" s="4" t="n">
         <v>21.2</v>
       </c>
-      <c r="L65" s="4" t="n">
+      <c r="M65" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -37534,14 +37739,17 @@
         <v>27.62</v>
       </c>
       <c r="K66" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L66" t="n">
         <v>11.08</v>
       </c>
-      <c r="L66" t="n">
+      <c r="M66" t="n">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <conditionalFormatting sqref="H2:H66">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -37590,6 +37798,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L66">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>